<commit_message>
Update Bloomberg inputs to forward P-E
</commit_message>
<xml_diff>
--- a/ibovespa_msci_return_decomposition/bloomberg_input_ibov_msci_brazil.xlsx
+++ b/ibovespa_msci_return_decomposition/bloomberg_input_ibov_msci_brazil.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -39,6 +39,10 @@
     <font>
       <b val="1"/>
       <color rgb="0017365D"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
@@ -75,16 +79,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,7 +501,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Bloomberg input — Ibovespa and MSCI Brazil</t>
+          <t>Bloomberg input - Ibovespa and MSCI Brazil - Forward P/E</t>
         </is>
       </c>
     </row>
@@ -542,33 +547,40 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Valuation basis: Bloomberg BEST_PE_RATIO with BEST_FPERIOD_OVERRIDE=1GY. Trailing PE_RATIO is not used.</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Series</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Total-return input</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Price-return input</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Dividend calculation</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Formula range</t>
         </is>
@@ -669,22 +681,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Latest date</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Required action</t>
         </is>
@@ -816,7 +828,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PE_RATIO</t>
+          <t>BEST_PE_RATIO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -832,7 +844,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <f t="array" ref="A7:E9006">_xll.BDH(B$4,B$6:E$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S")</f>
+        <f t="array" ref="A7:E9006">_xll.BDH(B$4,B$6:E$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S","BEST_FPERIOD_OVERRIDE=1GY")</f>
         <v/>
       </c>
       <c r="F7" s="1" t="n"/>
@@ -30082,12 +30094,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PE_RATIO</t>
+          <t>BEST_PE_RATIO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>TRAIL_12M_EPS</t>
+          <t>BEST_EPS</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -30107,22 +30119,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>PE_RATIO</t>
+          <t>BEST_PE_RATIO</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>TRAIL_12M_EPS</t>
+          <t>BEST_EPS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <f t="array" ref="A7:E9006">_xll.BDH(B$4,B$6:E$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S")</f>
+        <f t="array" ref="A7:E9006">_xll.BDH(B$4,B$6:E$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S","BEST_FPERIOD_OVERRIDE=1GY")</f>
         <v/>
       </c>
       <c r="F7" s="1">
-        <f t="array" ref="F7:J9006">_xll.BDH(G$4,G$6:J$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S")</f>
+        <f t="array" ref="F7:J9006">_xll.BDH(G$4,G$6:J$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S","BEST_FPERIOD_OVERRIDE=1GY")</f>
         <v/>
       </c>
     </row>

</xml_diff>